<commit_message>
Identify business in conditional formatting
</commit_message>
<xml_diff>
--- a/Arithmatics function.xlsx
+++ b/Arithmatics function.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dmart sales Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8ADE4A7F-CDD5-4B57-A589-E114D8E377C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{437D9A4F-549A-4E5A-B60C-0F9520C3EE28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="3" activeTab="7" xr2:uid="{2B6E4641-DF59-45C7-A5BC-A0F90F324489}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="4" activeTab="9" xr2:uid="{2B6E4641-DF59-45C7-A5BC-A0F90F324489}"/>
   </bookViews>
   <sheets>
     <sheet name="Arithmatic function" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,9 @@
     <sheet name="New Range" sheetId="5" r:id="rId5"/>
     <sheet name="String Functions" sheetId="7" r:id="rId6"/>
     <sheet name="Date Function" sheetId="8" r:id="rId7"/>
-    <sheet name="Sheet3" sheetId="9" r:id="rId8"/>
+    <sheet name="Flash Fill" sheetId="9" r:id="rId8"/>
+    <sheet name="statics function" sheetId="10" r:id="rId9"/>
+    <sheet name="Sheet2" sheetId="11" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="New_ranage">'New Range'!$D$2:$D$10</definedName>
@@ -46,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="147">
   <si>
     <t>A</t>
   </si>
@@ -397,6 +399,96 @@
   </si>
   <si>
     <t>Mumbai</t>
+  </si>
+  <si>
+    <t>median</t>
+  </si>
+  <si>
+    <t>Function</t>
+  </si>
+  <si>
+    <t>formula</t>
+  </si>
+  <si>
+    <t>mean</t>
+  </si>
+  <si>
+    <t>(n+1)/2</t>
+  </si>
+  <si>
+    <t>sum of a</t>
+  </si>
+  <si>
+    <t>count of a</t>
+  </si>
+  <si>
+    <t>mode</t>
+  </si>
+  <si>
+    <t>variance</t>
+  </si>
+  <si>
+    <t>Deviation</t>
+  </si>
+  <si>
+    <t>squre deviation</t>
+  </si>
+  <si>
+    <t>Standard Deviation</t>
+  </si>
+  <si>
+    <t>Standand dev</t>
+  </si>
+  <si>
+    <t>sqr var</t>
+  </si>
+  <si>
+    <t>avg sqr value of deviation</t>
+  </si>
+  <si>
+    <t>s</t>
+  </si>
+  <si>
+    <t>Product 1</t>
+  </si>
+  <si>
+    <t>Product 2</t>
+  </si>
+  <si>
+    <t>Product 3</t>
+  </si>
+  <si>
+    <t>Product 4</t>
+  </si>
+  <si>
+    <t>Product 5</t>
+  </si>
+  <si>
+    <t>Product 6</t>
+  </si>
+  <si>
+    <t>Product 7</t>
+  </si>
+  <si>
+    <t>Product 8</t>
+  </si>
+  <si>
+    <t>JAN</t>
+  </si>
+  <si>
+    <t>FEB</t>
+  </si>
+  <si>
+    <t>MAR</t>
+  </si>
+  <si>
+    <t>APR</t>
+  </si>
+  <si>
+    <t>MAY</t>
+  </si>
+  <si>
+    <t>JUN</t>
   </si>
 </sst>
 </file>
@@ -460,7 +552,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -483,12 +575,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -502,12 +609,749 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="77">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1443,6 +2287,252 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52A6C511-5875-4BF4-ABB5-8CE6A36DE6EB}">
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="F1" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="G1" s="12" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="B2" s="13">
+        <v>7996</v>
+      </c>
+      <c r="C2" s="13">
+        <v>7670</v>
+      </c>
+      <c r="D2" s="13">
+        <v>5958</v>
+      </c>
+      <c r="E2" s="13">
+        <v>8668</v>
+      </c>
+      <c r="F2" s="13">
+        <v>5793</v>
+      </c>
+      <c r="G2" s="13">
+        <v>9007</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="B3" s="13">
+        <v>7733</v>
+      </c>
+      <c r="C3" s="13">
+        <v>8542</v>
+      </c>
+      <c r="D3" s="13">
+        <v>6595</v>
+      </c>
+      <c r="E3" s="13">
+        <v>9923</v>
+      </c>
+      <c r="F3" s="13">
+        <v>7904</v>
+      </c>
+      <c r="G3" s="13">
+        <v>8684</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="B4" s="13">
+        <v>6243</v>
+      </c>
+      <c r="C4" s="13">
+        <v>5742</v>
+      </c>
+      <c r="D4" s="13">
+        <v>8364</v>
+      </c>
+      <c r="E4" s="13">
+        <v>7023</v>
+      </c>
+      <c r="F4" s="13">
+        <v>8859</v>
+      </c>
+      <c r="G4" s="13">
+        <v>8864</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="B5" s="13">
+        <v>8178</v>
+      </c>
+      <c r="C5" s="13">
+        <v>9617</v>
+      </c>
+      <c r="D5" s="13">
+        <v>7184</v>
+      </c>
+      <c r="E5" s="13">
+        <v>5908</v>
+      </c>
+      <c r="F5" s="13">
+        <v>6767</v>
+      </c>
+      <c r="G5" s="13">
+        <v>5127</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="13" t="s">
+        <v>137</v>
+      </c>
+      <c r="B6" s="13">
+        <v>7365</v>
+      </c>
+      <c r="C6" s="13">
+        <v>6437</v>
+      </c>
+      <c r="D6" s="13">
+        <v>6269</v>
+      </c>
+      <c r="E6" s="13">
+        <v>9146</v>
+      </c>
+      <c r="F6" s="13">
+        <v>9754</v>
+      </c>
+      <c r="G6" s="13">
+        <v>7967</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="B7" s="13">
+        <v>6200</v>
+      </c>
+      <c r="C7" s="13">
+        <v>7679</v>
+      </c>
+      <c r="D7" s="13">
+        <v>7432</v>
+      </c>
+      <c r="E7" s="13">
+        <v>9952</v>
+      </c>
+      <c r="F7" s="13">
+        <v>5549</v>
+      </c>
+      <c r="G7" s="13">
+        <v>9450</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="B8" s="13">
+        <v>9642</v>
+      </c>
+      <c r="C8" s="13">
+        <v>6213</v>
+      </c>
+      <c r="D8" s="13">
+        <v>5456</v>
+      </c>
+      <c r="E8" s="13">
+        <v>7775</v>
+      </c>
+      <c r="F8" s="13">
+        <v>7670</v>
+      </c>
+      <c r="G8" s="13">
+        <v>8877</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="13" t="s">
+        <v>140</v>
+      </c>
+      <c r="B9" s="13">
+        <v>9627</v>
+      </c>
+      <c r="C9" s="13">
+        <v>6309</v>
+      </c>
+      <c r="D9" s="13">
+        <v>5145</v>
+      </c>
+      <c r="E9" s="13">
+        <v>7611</v>
+      </c>
+      <c r="F9" s="13">
+        <v>6199</v>
+      </c>
+      <c r="G9" s="13">
+        <v>7813</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
+  <conditionalFormatting sqref="B2:G9">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFFF0000"/>
+        <color rgb="FF0070C0"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="10"/>
+        <color theme="4"/>
+        <color rgb="FF7030A0"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="num" val="6000"/>
+        <cfvo type="num" val="9000"/>
+        <color rgb="FFFF7128"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90054B61-6E1D-4DFD-A461-B11114C2B8F0}">
   <dimension ref="A1:I15"/>
@@ -2489,7 +3579,7 @@
       </c>
       <c r="B1" s="6">
         <f ca="1">TODAY()</f>
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="C1" s="5"/>
     </row>
@@ -2499,7 +3589,7 @@
       </c>
       <c r="B2" s="7">
         <f ca="1">NOW()</f>
-        <v>46324.51853321759</v>
+        <v>46325.513034143522</v>
       </c>
       <c r="C2" s="5"/>
     </row>
@@ -2519,7 +3609,7 @@
       </c>
       <c r="B4" s="5">
         <f ca="1">DAY(B1)</f>
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C4" s="5"/>
     </row>
@@ -2540,7 +3630,7 @@
       </c>
       <c r="B6" s="5">
         <f ca="1">WEEKDAY(B1,11)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C6" s="5"/>
     </row>
@@ -2570,7 +3660,7 @@
       <c r="A9" s="5"/>
       <c r="B9" s="5" t="str">
         <f ca="1">TEXT(TODAY(),"DDDD")</f>
-        <v>Thursday</v>
+        <v>Friday</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>87</v>
@@ -2582,7 +3672,7 @@
       </c>
       <c r="C11" s="3">
         <f ca="1">TODAY()</f>
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="D11" s="4"/>
       <c r="E11" s="4">
@@ -2613,7 +3703,7 @@
       <c r="D13" s="4"/>
       <c r="E13" s="4">
         <f ca="1">DATEDIF(B11,C11,"D")</f>
-        <v>1387</v>
+        <v>1388</v>
       </c>
       <c r="F13" s="4" t="s">
         <v>90</v>
@@ -2626,7 +3716,7 @@
       </c>
       <c r="B15" s="2">
         <f ca="1">EDATE(B1,6)</f>
-        <v>46506</v>
+        <v>46507</v>
       </c>
     </row>
   </sheetData>
@@ -2798,4 +3888,317 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3ED12DB4-ECF0-47AD-9D46-3FFDEC5DF6B2}">
+  <dimension ref="A1:K18"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="10" max="10" width="15" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="I1" t="s">
+        <v>126</v>
+      </c>
+      <c r="J1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>31</v>
+      </c>
+      <c r="D2" t="s">
+        <v>118</v>
+      </c>
+      <c r="E2" t="s">
+        <v>119</v>
+      </c>
+      <c r="I2">
+        <f>A2-D4</f>
+        <v>-20.714285714285715</v>
+      </c>
+      <c r="J2">
+        <f>I2^2</f>
+        <v>429.08163265306126</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>33</v>
+      </c>
+      <c r="F3" t="s">
+        <v>122</v>
+      </c>
+      <c r="G3" t="s">
+        <v>123</v>
+      </c>
+      <c r="I3">
+        <f>A3-D4</f>
+        <v>-18.714285714285715</v>
+      </c>
+      <c r="J3">
+        <f t="shared" ref="J3:J15" si="0">I3^2</f>
+        <v>350.22448979591843</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>37</v>
+      </c>
+      <c r="C4" t="s">
+        <v>120</v>
+      </c>
+      <c r="D4">
+        <f>AVERAGE(A2:A15)</f>
+        <v>51.714285714285715</v>
+      </c>
+      <c r="E4">
+        <f>F4/G4</f>
+        <v>51.714285714285715</v>
+      </c>
+      <c r="F4">
+        <f>SUM(A2:A15)</f>
+        <v>724</v>
+      </c>
+      <c r="G4">
+        <v>14</v>
+      </c>
+      <c r="I4">
+        <f>A4-D4</f>
+        <v>-14.714285714285715</v>
+      </c>
+      <c r="J4">
+        <f t="shared" si="0"/>
+        <v>216.51020408163268</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>37</v>
+      </c>
+      <c r="I5">
+        <f>A5-E4</f>
+        <v>-14.714285714285715</v>
+      </c>
+      <c r="J5">
+        <f t="shared" si="0"/>
+        <v>216.51020408163268</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>43</v>
+      </c>
+      <c r="E6" t="s">
+        <v>121</v>
+      </c>
+      <c r="I6">
+        <f>A6-D4</f>
+        <v>-8.7142857142857153</v>
+      </c>
+      <c r="J6">
+        <f t="shared" si="0"/>
+        <v>75.938775510204096</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>43</v>
+      </c>
+      <c r="C7" t="s">
+        <v>117</v>
+      </c>
+      <c r="D7">
+        <f>MEDIAN(A2:A15)</f>
+        <v>45.5</v>
+      </c>
+      <c r="E7">
+        <f>(14+1)/2</f>
+        <v>7.5</v>
+      </c>
+      <c r="I7">
+        <f>A7-D4</f>
+        <v>-8.7142857142857153</v>
+      </c>
+      <c r="J7">
+        <f t="shared" si="0"/>
+        <v>75.938775510204096</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>45</v>
+      </c>
+      <c r="I8">
+        <f>A8-D4</f>
+        <v>-6.7142857142857153</v>
+      </c>
+      <c r="J8">
+        <f t="shared" si="0"/>
+        <v>45.081632653061241</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>46</v>
+      </c>
+      <c r="C9" t="s">
+        <v>124</v>
+      </c>
+      <c r="D9">
+        <f>_xlfn.MODE.SNGL(A2:A15)</f>
+        <v>37</v>
+      </c>
+      <c r="I9">
+        <f>A9-E4</f>
+        <v>-5.7142857142857153</v>
+      </c>
+      <c r="J9">
+        <f t="shared" si="0"/>
+        <v>32.653061224489811</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>52</v>
+      </c>
+      <c r="D10">
+        <f t="array" ref="D10:D13">_xlfn.MODE.MULT(A4:A15)</f>
+        <v>37</v>
+      </c>
+      <c r="I10">
+        <f>A10-E4</f>
+        <v>0.2857142857142847</v>
+      </c>
+      <c r="J10">
+        <f t="shared" si="0"/>
+        <v>8.1632653061223914E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>52</v>
+      </c>
+      <c r="D11">
+        <v>43</v>
+      </c>
+      <c r="I11">
+        <f>A11-E4</f>
+        <v>0.2857142857142847</v>
+      </c>
+      <c r="J11">
+        <f t="shared" si="0"/>
+        <v>8.1632653061223914E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>62</v>
+      </c>
+      <c r="D12">
+        <v>52</v>
+      </c>
+      <c r="I12">
+        <f>A12-D4</f>
+        <v>10.285714285714285</v>
+      </c>
+      <c r="J12">
+        <f t="shared" si="0"/>
+        <v>105.79591836734691</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>70</v>
+      </c>
+      <c r="D13" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I13">
+        <f>A13-E4</f>
+        <v>18.285714285714285</v>
+      </c>
+      <c r="J13">
+        <f t="shared" si="0"/>
+        <v>334.36734693877548</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>81</v>
+      </c>
+      <c r="C14" t="s">
+        <v>125</v>
+      </c>
+      <c r="D14">
+        <f>AVERAGE(J2:J15)</f>
+        <v>311.63265306122452</v>
+      </c>
+      <c r="E14" t="s">
+        <v>131</v>
+      </c>
+      <c r="I14">
+        <f>A14-E4</f>
+        <v>29.285714285714285</v>
+      </c>
+      <c r="J14">
+        <f t="shared" si="0"/>
+        <v>857.65306122448976</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>92</v>
+      </c>
+      <c r="I15">
+        <f>A15-E4</f>
+        <v>40.285714285714285</v>
+      </c>
+      <c r="J15">
+        <f t="shared" si="0"/>
+        <v>1622.9387755102041</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C16" t="s">
+        <v>128</v>
+      </c>
+      <c r="E16">
+        <f>_xlfn.STDEV.P(A2:A15)</f>
+        <v>17.653120207522083</v>
+      </c>
+      <c r="F16" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="17" spans="10:11" x14ac:dyDescent="0.25">
+      <c r="J17" t="s">
+        <v>129</v>
+      </c>
+      <c r="K17" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="18" spans="10:11" x14ac:dyDescent="0.25">
+      <c r="J18">
+        <f>_xlfn.VAR.P(A2:A15)</f>
+        <v>311.63265306122452</v>
+      </c>
+      <c r="K18">
+        <f>SQRT(J18)</f>
+        <v>17.653120207522083</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:A15">
+    <sortCondition ref="A2:A15"/>
+  </sortState>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>